<commit_message>
Upgraded E2E Reporting Engine to Custom OpenPyXL Dashboard UI and added React Native Student App
</commit_message>
<xml_diff>
--- a/backend/E2E_Test_Report.xlsx
+++ b/backend/E2E_Test_Report.xlsx
@@ -453,7 +453,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-06-15 16:36:24</t>
+          <t>2026-06-15 17:15:52</t>
         </is>
       </c>
     </row>
@@ -654,7 +654,7 @@
         </is>
       </c>
       <c r="F2" t="n">
-        <v>2.19</v>
+        <v>2.26</v>
       </c>
       <c r="G2" t="inlineStr"/>
     </row>
@@ -685,7 +685,7 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>1.08</v>
+        <v>2.85</v>
       </c>
       <c r="G3" t="inlineStr"/>
     </row>
@@ -716,7 +716,7 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>1.37</v>
+        <v>8.06</v>
       </c>
       <c r="G4" t="inlineStr"/>
     </row>
@@ -747,7 +747,7 @@
         </is>
       </c>
       <c r="F5" t="n">
-        <v>1.49</v>
+        <v>2.35</v>
       </c>
       <c r="G5" t="inlineStr"/>
     </row>
@@ -778,7 +778,7 @@
         </is>
       </c>
       <c r="F6" t="n">
-        <v>2.57</v>
+        <v>1.79</v>
       </c>
       <c r="G6" t="inlineStr"/>
     </row>
@@ -809,7 +809,7 @@
         </is>
       </c>
       <c r="F7" t="n">
-        <v>1.62</v>
+        <v>1.89</v>
       </c>
       <c r="G7" t="inlineStr"/>
     </row>
@@ -840,7 +840,7 @@
         </is>
       </c>
       <c r="F8" t="n">
-        <v>1.63</v>
+        <v>1.9</v>
       </c>
       <c r="G8" t="inlineStr"/>
     </row>
@@ -871,7 +871,7 @@
         </is>
       </c>
       <c r="F9" t="n">
-        <v>2.65</v>
+        <v>2.06</v>
       </c>
       <c r="G9" t="inlineStr"/>
     </row>
@@ -902,7 +902,7 @@
         </is>
       </c>
       <c r="F10" t="n">
-        <v>2.83</v>
+        <v>1.88</v>
       </c>
       <c r="G10" t="inlineStr"/>
     </row>
@@ -933,7 +933,7 @@
         </is>
       </c>
       <c r="F11" t="n">
-        <v>2.05</v>
+        <v>2.01</v>
       </c>
       <c r="G11" t="inlineStr"/>
     </row>
@@ -964,7 +964,7 @@
         </is>
       </c>
       <c r="F12" t="n">
-        <v>1.32</v>
+        <v>1.5</v>
       </c>
       <c r="G12" t="inlineStr"/>
     </row>
@@ -995,7 +995,7 @@
         </is>
       </c>
       <c r="F13" t="n">
-        <v>1.63</v>
+        <v>2.14</v>
       </c>
       <c r="G13" t="inlineStr"/>
     </row>
@@ -1026,7 +1026,7 @@
         </is>
       </c>
       <c r="F14" t="n">
-        <v>1.46</v>
+        <v>1.36</v>
       </c>
       <c r="G14" t="inlineStr"/>
     </row>
@@ -1057,7 +1057,7 @@
         </is>
       </c>
       <c r="F15" t="n">
-        <v>1.53</v>
+        <v>2.2</v>
       </c>
       <c r="G15" t="inlineStr"/>
     </row>
@@ -1088,7 +1088,7 @@
         </is>
       </c>
       <c r="F16" t="n">
-        <v>3.44</v>
+        <v>1.76</v>
       </c>
       <c r="G16" t="inlineStr"/>
     </row>
@@ -1119,7 +1119,7 @@
         </is>
       </c>
       <c r="F17" t="n">
-        <v>1.71</v>
+        <v>1.38</v>
       </c>
       <c r="G17" t="inlineStr"/>
     </row>
@@ -1150,7 +1150,7 @@
         </is>
       </c>
       <c r="F18" t="n">
-        <v>2.83</v>
+        <v>1.99</v>
       </c>
       <c r="G18" t="inlineStr"/>
     </row>
@@ -1181,7 +1181,7 @@
         </is>
       </c>
       <c r="F19" t="n">
-        <v>1.62</v>
+        <v>1.98</v>
       </c>
       <c r="G19" t="inlineStr"/>
     </row>
@@ -1212,7 +1212,7 @@
         </is>
       </c>
       <c r="F20" t="n">
-        <v>1.54</v>
+        <v>1.75</v>
       </c>
       <c r="G20" t="inlineStr"/>
     </row>
@@ -1274,7 +1274,7 @@
         </is>
       </c>
       <c r="F22" t="n">
-        <v>1.87</v>
+        <v>2.38</v>
       </c>
       <c r="G22" t="inlineStr"/>
     </row>
@@ -1305,7 +1305,7 @@
         </is>
       </c>
       <c r="F23" t="n">
-        <v>1.81</v>
+        <v>2.05</v>
       </c>
       <c r="G23" t="inlineStr"/>
     </row>
@@ -1336,7 +1336,7 @@
         </is>
       </c>
       <c r="F24" t="n">
-        <v>1.61</v>
+        <v>1.3</v>
       </c>
       <c r="G24" t="inlineStr"/>
     </row>
@@ -1367,7 +1367,7 @@
         </is>
       </c>
       <c r="F25" t="n">
-        <v>2</v>
+        <v>1.82</v>
       </c>
       <c r="G25" t="inlineStr"/>
     </row>
@@ -1398,7 +1398,7 @@
         </is>
       </c>
       <c r="F26" t="n">
-        <v>2.07</v>
+        <v>2.19</v>
       </c>
       <c r="G26" t="inlineStr"/>
     </row>
@@ -1429,7 +1429,7 @@
         </is>
       </c>
       <c r="F27" t="n">
-        <v>2.91</v>
+        <v>1.26</v>
       </c>
       <c r="G27" t="inlineStr"/>
     </row>
@@ -2545,7 +2545,7 @@
         </is>
       </c>
       <c r="F63" t="n">
-        <v>0.68</v>
+        <v>0.7</v>
       </c>
       <c r="G63" t="inlineStr"/>
     </row>
@@ -2576,7 +2576,7 @@
         </is>
       </c>
       <c r="F64" t="n">
-        <v>0.62</v>
+        <v>0.85</v>
       </c>
       <c r="G64" t="inlineStr"/>
     </row>
@@ -2607,7 +2607,7 @@
         </is>
       </c>
       <c r="F65" t="n">
-        <v>0.6</v>
+        <v>0.76</v>
       </c>
       <c r="G65" t="inlineStr"/>
     </row>
@@ -2638,7 +2638,7 @@
         </is>
       </c>
       <c r="F66" t="n">
-        <v>0.57</v>
+        <v>0.62</v>
       </c>
       <c r="G66" t="inlineStr"/>
     </row>
@@ -2669,7 +2669,7 @@
         </is>
       </c>
       <c r="F67" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="G67" t="inlineStr"/>
     </row>
@@ -2700,7 +2700,7 @@
         </is>
       </c>
       <c r="F68" t="n">
-        <v>0.91</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="G68" t="inlineStr"/>
     </row>
@@ -2731,7 +2731,7 @@
         </is>
       </c>
       <c r="F69" t="n">
-        <v>0.63</v>
+        <v>0.61</v>
       </c>
       <c r="G69" t="inlineStr"/>
     </row>
@@ -2762,7 +2762,7 @@
         </is>
       </c>
       <c r="F70" t="n">
-        <v>0.6</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="G70" t="inlineStr"/>
     </row>
@@ -2793,7 +2793,7 @@
         </is>
       </c>
       <c r="F71" t="n">
-        <v>0.64</v>
+        <v>0.73</v>
       </c>
       <c r="G71" t="inlineStr"/>
     </row>
@@ -2824,7 +2824,7 @@
         </is>
       </c>
       <c r="F72" t="n">
-        <v>0.67</v>
+        <v>0.64</v>
       </c>
       <c r="G72" t="inlineStr"/>
     </row>
@@ -2855,7 +2855,7 @@
         </is>
       </c>
       <c r="F73" t="n">
-        <v>0.67</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="G73" t="inlineStr"/>
     </row>
@@ -2886,7 +2886,7 @@
         </is>
       </c>
       <c r="F74" t="n">
-        <v>0.67</v>
+        <v>0.78</v>
       </c>
       <c r="G74" t="inlineStr"/>
     </row>
@@ -2917,7 +2917,7 @@
         </is>
       </c>
       <c r="F75" t="n">
-        <v>0.7</v>
+        <v>0.61</v>
       </c>
       <c r="G75" t="inlineStr"/>
     </row>
@@ -2948,7 +2948,7 @@
         </is>
       </c>
       <c r="F76" t="n">
-        <v>0.67</v>
+        <v>1.09</v>
       </c>
       <c r="G76" t="inlineStr"/>
     </row>
@@ -2979,7 +2979,7 @@
         </is>
       </c>
       <c r="F77" t="n">
-        <v>0.66</v>
+        <v>1.29</v>
       </c>
       <c r="G77" t="inlineStr"/>
     </row>
@@ -3010,7 +3010,7 @@
         </is>
       </c>
       <c r="F78" t="n">
-        <v>0.58</v>
+        <v>0.99</v>
       </c>
       <c r="G78" t="inlineStr"/>
     </row>
@@ -3041,7 +3041,7 @@
         </is>
       </c>
       <c r="F79" t="n">
-        <v>0.68</v>
+        <v>0.78</v>
       </c>
       <c r="G79" t="inlineStr"/>
     </row>
@@ -3072,7 +3072,7 @@
         </is>
       </c>
       <c r="F80" t="n">
-        <v>0.62</v>
+        <v>0.83</v>
       </c>
       <c r="G80" t="inlineStr"/>
     </row>
@@ -3103,7 +3103,7 @@
         </is>
       </c>
       <c r="F81" t="n">
-        <v>0.82</v>
+        <v>1.06</v>
       </c>
       <c r="G81" t="inlineStr"/>
     </row>
@@ -3134,7 +3134,7 @@
         </is>
       </c>
       <c r="F82" t="n">
-        <v>0.62</v>
+        <v>0.87</v>
       </c>
       <c r="G82" t="inlineStr"/>
     </row>
@@ -3165,7 +3165,7 @@
         </is>
       </c>
       <c r="F83" t="n">
-        <v>0.62</v>
+        <v>0.78</v>
       </c>
       <c r="G83" t="inlineStr"/>
     </row>
@@ -3196,7 +3196,7 @@
         </is>
       </c>
       <c r="F84" t="n">
-        <v>0.83</v>
+        <v>0.89</v>
       </c>
       <c r="G84" t="inlineStr"/>
     </row>
@@ -3227,7 +3227,7 @@
         </is>
       </c>
       <c r="F85" t="n">
-        <v>0.6</v>
+        <v>1.1</v>
       </c>
       <c r="G85" t="inlineStr"/>
     </row>
@@ -3258,7 +3258,7 @@
         </is>
       </c>
       <c r="F86" t="n">
-        <v>0.75</v>
+        <v>0.77</v>
       </c>
       <c r="G86" t="inlineStr"/>
     </row>
@@ -3289,7 +3289,7 @@
         </is>
       </c>
       <c r="F87" t="n">
-        <v>1.67</v>
+        <v>0.76</v>
       </c>
       <c r="G87" t="inlineStr"/>
     </row>
@@ -3320,7 +3320,7 @@
         </is>
       </c>
       <c r="F88" t="n">
-        <v>0.9</v>
+        <v>0.85</v>
       </c>
       <c r="G88" t="inlineStr"/>
     </row>
@@ -3351,7 +3351,7 @@
         </is>
       </c>
       <c r="F89" t="n">
-        <v>1.08</v>
+        <v>0.65</v>
       </c>
       <c r="G89" t="inlineStr"/>
     </row>
@@ -3382,7 +3382,7 @@
         </is>
       </c>
       <c r="F90" t="n">
-        <v>0.77</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="G90" t="inlineStr"/>
     </row>
@@ -3413,7 +3413,7 @@
         </is>
       </c>
       <c r="F91" t="n">
-        <v>0.79</v>
+        <v>0.91</v>
       </c>
       <c r="G91" t="inlineStr"/>
     </row>
@@ -3444,7 +3444,7 @@
         </is>
       </c>
       <c r="F92" t="n">
-        <v>0.92</v>
+        <v>0.84</v>
       </c>
       <c r="G92" t="inlineStr"/>
     </row>
@@ -3475,7 +3475,7 @@
         </is>
       </c>
       <c r="F93" t="n">
-        <v>1.03</v>
+        <v>0.98</v>
       </c>
       <c r="G93" t="inlineStr"/>
     </row>
@@ -3506,7 +3506,7 @@
         </is>
       </c>
       <c r="F94" t="n">
-        <v>1.55</v>
+        <v>0.67</v>
       </c>
       <c r="G94" t="inlineStr"/>
     </row>
@@ -3537,7 +3537,7 @@
         </is>
       </c>
       <c r="F95" t="n">
-        <v>1.45</v>
+        <v>0.76</v>
       </c>
       <c r="G95" t="inlineStr"/>
     </row>
@@ -3568,7 +3568,7 @@
         </is>
       </c>
       <c r="F96" t="n">
-        <v>1.36</v>
+        <v>0.93</v>
       </c>
       <c r="G96" t="inlineStr"/>
     </row>
@@ -3599,7 +3599,7 @@
         </is>
       </c>
       <c r="F97" t="n">
-        <v>0.68</v>
+        <v>0.79</v>
       </c>
       <c r="G97" t="inlineStr"/>
     </row>
@@ -3630,7 +3630,7 @@
         </is>
       </c>
       <c r="F98" t="n">
-        <v>0.6</v>
+        <v>0.7</v>
       </c>
       <c r="G98" t="inlineStr"/>
     </row>
@@ -3661,7 +3661,7 @@
         </is>
       </c>
       <c r="F99" t="n">
-        <v>0.63</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="G99" t="inlineStr"/>
     </row>
@@ -3692,7 +3692,7 @@
         </is>
       </c>
       <c r="F100" t="n">
-        <v>0.71</v>
+        <v>0.85</v>
       </c>
       <c r="G100" t="inlineStr"/>
     </row>
@@ -3723,7 +3723,7 @@
         </is>
       </c>
       <c r="F101" t="n">
-        <v>0.84</v>
+        <v>0.77</v>
       </c>
       <c r="G101" t="inlineStr"/>
     </row>
@@ -3754,7 +3754,7 @@
         </is>
       </c>
       <c r="F102" t="n">
-        <v>0.67</v>
+        <v>0.74</v>
       </c>
       <c r="G102" t="inlineStr"/>
     </row>
@@ -3785,7 +3785,7 @@
         </is>
       </c>
       <c r="F103" t="n">
-        <v>0.63</v>
+        <v>0.71</v>
       </c>
       <c r="G103" t="inlineStr"/>
     </row>
@@ -3816,7 +3816,7 @@
         </is>
       </c>
       <c r="F104" t="n">
-        <v>1.91</v>
+        <v>0.67</v>
       </c>
       <c r="G104" t="inlineStr"/>
     </row>
@@ -3847,7 +3847,7 @@
         </is>
       </c>
       <c r="F105" t="n">
-        <v>0</v>
+        <v>0.01</v>
       </c>
       <c r="G105" t="inlineStr"/>
     </row>
@@ -3909,7 +3909,7 @@
         </is>
       </c>
       <c r="F107" t="n">
-        <v>0.77</v>
+        <v>1.18</v>
       </c>
       <c r="G107" t="inlineStr"/>
     </row>
@@ -3940,7 +3940,7 @@
         </is>
       </c>
       <c r="F108" t="n">
-        <v>2.16</v>
+        <v>4.63</v>
       </c>
       <c r="G108" t="inlineStr"/>
     </row>

</xml_diff>

<commit_message>
Updated mobile app API endpoint to use live Render server and updated README links
</commit_message>
<xml_diff>
--- a/backend/E2E_Test_Report.xlsx
+++ b/backend/E2E_Test_Report.xlsx
@@ -18,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -26,16 +26,72 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="16"/>
+    </font>
+    <font>
+      <b val="1"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00385723"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="001F497D"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="001F497D"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="001F497D"/>
+      <sz val="24"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00385723"/>
+      <sz val="24"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F497D"/>
+        <bgColor rgb="001F497D"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E2EFDA"/>
+        <bgColor rgb="00E2EFDA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F2F2F2"/>
+        <bgColor rgb="00F2F2F2"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -43,12 +99,54 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -414,160 +512,282 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B13"/>
+  <dimension ref="A1:E21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
-    <col width="50" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>Metric</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>Value</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Project Title</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>SecureExam - Automated E2E Testing Report</t>
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>SECUREEXAM APP - QA E2E TEST REPORT</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Execution Date</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>2026-06-15 17:15:52</t>
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Test Run Date:</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-16</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Deployable Status</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>READY FOR DEPLOYMENT ✅</t>
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Test Run Time:</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>09:58:27</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Total Test Cases</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>OS / Platform:</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Windows / Python Test Server</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>App Version Name:</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>1.0 (Universal)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Deployable Status:</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>DEPLOYABLE - FIT FOR RELEASE</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>Core Metrics KPI Summary</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="6" t="inlineStr">
+        <is>
+          <t>TOTAL TEST CASES</t>
+        </is>
+      </c>
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="C11" s="6" t="inlineStr">
+        <is>
+          <t>FAILED</t>
+        </is>
+      </c>
+      <c r="D11" s="6" t="inlineStr">
+        <is>
+          <t>PASS RATE</t>
+        </is>
+      </c>
+      <c r="E11" s="6" t="inlineStr">
+        <is>
+          <t>DURATION (SEC)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="40" customHeight="1">
+      <c r="A12" s="7" t="n">
         <v>107</v>
       </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Passed Test Cases</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
+      <c r="B12" s="8" t="n">
         <v>107</v>
       </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Failed Test Cases</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
+      <c r="C12" s="7" t="n">
         <v>0</v>
       </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
+      <c r="D12" s="7" t="inlineStr">
+        <is>
+          <t>100.0%</t>
+        </is>
+      </c>
+      <c r="E12" s="7" t="inlineStr">
+        <is>
+          <t>176.67</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>Category-Wise Execution Breakdown</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="9" t="inlineStr">
+        <is>
+          <t>Test Category</t>
+        </is>
+      </c>
+      <c r="B16" s="10" t="inlineStr">
+        <is>
+          <t>Total Cases</t>
+        </is>
+      </c>
+      <c r="C16" s="10" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="D16" s="10" t="inlineStr">
+        <is>
+          <t>Failed</t>
+        </is>
+      </c>
+      <c r="E16" s="10" t="inlineStr">
         <is>
           <t>Pass Rate</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+    </row>
+    <row r="17">
+      <c r="A17" s="11" t="inlineStr">
+        <is>
+          <t>Validation Test</t>
+        </is>
+      </c>
+      <c r="B17" s="12" t="n">
+        <v>31</v>
+      </c>
+      <c r="C17" s="12" t="n">
+        <v>31</v>
+      </c>
+      <c r="D17" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="E17" s="12" t="inlineStr">
         <is>
           <t>100.0%</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>-- BREAKDOWN BY CATEGORY --</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr"/>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
+    <row r="18">
+      <c r="A18" s="11" t="inlineStr">
+        <is>
+          <t>UI/UX Test</t>
+        </is>
+      </c>
+      <c r="B18" s="12" t="n">
+        <v>10</v>
+      </c>
+      <c r="C18" s="12" t="n">
+        <v>10</v>
+      </c>
+      <c r="D18" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="E18" s="12" t="inlineStr">
+        <is>
+          <t>100.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="11" t="inlineStr">
+        <is>
+          <t>Functional Testing</t>
+        </is>
+      </c>
+      <c r="B19" s="12" t="n">
+        <v>62</v>
+      </c>
+      <c r="C19" s="12" t="n">
+        <v>62</v>
+      </c>
+      <c r="D19" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="E19" s="12" t="inlineStr">
+        <is>
+          <t>100.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="11" t="inlineStr">
         <is>
           <t>Unit Testing</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>4/4 Passed</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>UI/UX Test</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>10/10 Passed</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>Functional Testing</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>62/62 Passed</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>Validation Test</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>31/31 Passed</t>
+      <c r="B20" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="C20" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="D20" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="E20" s="12" t="inlineStr">
+        <is>
+          <t>100.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="13" t="inlineStr">
+        <is>
+          <t>Total Summary</t>
+        </is>
+      </c>
+      <c r="B21" s="14" t="n">
+        <v>107</v>
+      </c>
+      <c r="C21" s="14" t="n">
+        <v>107</v>
+      </c>
+      <c r="D21" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="E21" s="14" t="inlineStr">
+        <is>
+          <t>100.0%</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="B7:E7"/>
+    <mergeCell ref="A1:E1"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -654,7 +874,7 @@
         </is>
       </c>
       <c r="F2" t="n">
-        <v>2.26</v>
+        <v>2.22</v>
       </c>
       <c r="G2" t="inlineStr"/>
     </row>
@@ -685,7 +905,7 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>2.85</v>
+        <v>2.06</v>
       </c>
       <c r="G3" t="inlineStr"/>
     </row>
@@ -716,7 +936,7 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>8.06</v>
+        <v>12.62</v>
       </c>
       <c r="G4" t="inlineStr"/>
     </row>
@@ -747,7 +967,7 @@
         </is>
       </c>
       <c r="F5" t="n">
-        <v>2.35</v>
+        <v>1.6</v>
       </c>
       <c r="G5" t="inlineStr"/>
     </row>
@@ -778,7 +998,7 @@
         </is>
       </c>
       <c r="F6" t="n">
-        <v>1.79</v>
+        <v>2.64</v>
       </c>
       <c r="G6" t="inlineStr"/>
     </row>
@@ -809,7 +1029,7 @@
         </is>
       </c>
       <c r="F7" t="n">
-        <v>1.89</v>
+        <v>1.65</v>
       </c>
       <c r="G7" t="inlineStr"/>
     </row>
@@ -840,7 +1060,7 @@
         </is>
       </c>
       <c r="F8" t="n">
-        <v>1.9</v>
+        <v>1.19</v>
       </c>
       <c r="G8" t="inlineStr"/>
     </row>
@@ -871,7 +1091,7 @@
         </is>
       </c>
       <c r="F9" t="n">
-        <v>2.06</v>
+        <v>1.6</v>
       </c>
       <c r="G9" t="inlineStr"/>
     </row>
@@ -902,7 +1122,7 @@
         </is>
       </c>
       <c r="F10" t="n">
-        <v>1.88</v>
+        <v>3.05</v>
       </c>
       <c r="G10" t="inlineStr"/>
     </row>
@@ -933,7 +1153,7 @@
         </is>
       </c>
       <c r="F11" t="n">
-        <v>2.01</v>
+        <v>2.53</v>
       </c>
       <c r="G11" t="inlineStr"/>
     </row>
@@ -964,7 +1184,7 @@
         </is>
       </c>
       <c r="F12" t="n">
-        <v>1.5</v>
+        <v>1.44</v>
       </c>
       <c r="G12" t="inlineStr"/>
     </row>
@@ -995,7 +1215,7 @@
         </is>
       </c>
       <c r="F13" t="n">
-        <v>2.14</v>
+        <v>1.88</v>
       </c>
       <c r="G13" t="inlineStr"/>
     </row>
@@ -1026,7 +1246,7 @@
         </is>
       </c>
       <c r="F14" t="n">
-        <v>1.36</v>
+        <v>1.66</v>
       </c>
       <c r="G14" t="inlineStr"/>
     </row>
@@ -1057,7 +1277,7 @@
         </is>
       </c>
       <c r="F15" t="n">
-        <v>2.2</v>
+        <v>1.97</v>
       </c>
       <c r="G15" t="inlineStr"/>
     </row>
@@ -1088,7 +1308,7 @@
         </is>
       </c>
       <c r="F16" t="n">
-        <v>1.76</v>
+        <v>1.99</v>
       </c>
       <c r="G16" t="inlineStr"/>
     </row>
@@ -1119,7 +1339,7 @@
         </is>
       </c>
       <c r="F17" t="n">
-        <v>1.38</v>
+        <v>2.5</v>
       </c>
       <c r="G17" t="inlineStr"/>
     </row>
@@ -1150,7 +1370,7 @@
         </is>
       </c>
       <c r="F18" t="n">
-        <v>1.99</v>
+        <v>2.9</v>
       </c>
       <c r="G18" t="inlineStr"/>
     </row>
@@ -1181,7 +1401,7 @@
         </is>
       </c>
       <c r="F19" t="n">
-        <v>1.98</v>
+        <v>2.55</v>
       </c>
       <c r="G19" t="inlineStr"/>
     </row>
@@ -1212,7 +1432,7 @@
         </is>
       </c>
       <c r="F20" t="n">
-        <v>1.75</v>
+        <v>2.45</v>
       </c>
       <c r="G20" t="inlineStr"/>
     </row>
@@ -1243,7 +1463,7 @@
         </is>
       </c>
       <c r="F21" t="n">
-        <v>1.51</v>
+        <v>1.73</v>
       </c>
       <c r="G21" t="inlineStr"/>
     </row>
@@ -1274,7 +1494,7 @@
         </is>
       </c>
       <c r="F22" t="n">
-        <v>2.38</v>
+        <v>2.72</v>
       </c>
       <c r="G22" t="inlineStr"/>
     </row>
@@ -1305,7 +1525,7 @@
         </is>
       </c>
       <c r="F23" t="n">
-        <v>2.05</v>
+        <v>2.54</v>
       </c>
       <c r="G23" t="inlineStr"/>
     </row>
@@ -1336,7 +1556,7 @@
         </is>
       </c>
       <c r="F24" t="n">
-        <v>1.3</v>
+        <v>1.46</v>
       </c>
       <c r="G24" t="inlineStr"/>
     </row>
@@ -1367,7 +1587,7 @@
         </is>
       </c>
       <c r="F25" t="n">
-        <v>1.82</v>
+        <v>1.26</v>
       </c>
       <c r="G25" t="inlineStr"/>
     </row>
@@ -1398,7 +1618,7 @@
         </is>
       </c>
       <c r="F26" t="n">
-        <v>2.19</v>
+        <v>2.64</v>
       </c>
       <c r="G26" t="inlineStr"/>
     </row>
@@ -1429,7 +1649,7 @@
         </is>
       </c>
       <c r="F27" t="n">
-        <v>1.26</v>
+        <v>2.18</v>
       </c>
       <c r="G27" t="inlineStr"/>
     </row>
@@ -2545,7 +2765,7 @@
         </is>
       </c>
       <c r="F63" t="n">
-        <v>0.7</v>
+        <v>2.03</v>
       </c>
       <c r="G63" t="inlineStr"/>
     </row>
@@ -2576,7 +2796,7 @@
         </is>
       </c>
       <c r="F64" t="n">
-        <v>0.85</v>
+        <v>2.26</v>
       </c>
       <c r="G64" t="inlineStr"/>
     </row>
@@ -2607,7 +2827,7 @@
         </is>
       </c>
       <c r="F65" t="n">
-        <v>0.76</v>
+        <v>1.61</v>
       </c>
       <c r="G65" t="inlineStr"/>
     </row>
@@ -2638,7 +2858,7 @@
         </is>
       </c>
       <c r="F66" t="n">
-        <v>0.62</v>
+        <v>1.67</v>
       </c>
       <c r="G66" t="inlineStr"/>
     </row>
@@ -2669,7 +2889,7 @@
         </is>
       </c>
       <c r="F67" t="n">
-        <v>0.9399999999999999</v>
+        <v>1.54</v>
       </c>
       <c r="G67" t="inlineStr"/>
     </row>
@@ -2700,7 +2920,7 @@
         </is>
       </c>
       <c r="F68" t="n">
-        <v>0.6899999999999999</v>
+        <v>1.06</v>
       </c>
       <c r="G68" t="inlineStr"/>
     </row>
@@ -2731,7 +2951,7 @@
         </is>
       </c>
       <c r="F69" t="n">
-        <v>0.61</v>
+        <v>1.26</v>
       </c>
       <c r="G69" t="inlineStr"/>
     </row>
@@ -2762,7 +2982,7 @@
         </is>
       </c>
       <c r="F70" t="n">
-        <v>0.6899999999999999</v>
+        <v>1.27</v>
       </c>
       <c r="G70" t="inlineStr"/>
     </row>
@@ -2793,7 +3013,7 @@
         </is>
       </c>
       <c r="F71" t="n">
-        <v>0.73</v>
+        <v>1.95</v>
       </c>
       <c r="G71" t="inlineStr"/>
     </row>
@@ -2824,7 +3044,7 @@
         </is>
       </c>
       <c r="F72" t="n">
-        <v>0.64</v>
+        <v>1.42</v>
       </c>
       <c r="G72" t="inlineStr"/>
     </row>
@@ -2855,7 +3075,7 @@
         </is>
       </c>
       <c r="F73" t="n">
-        <v>0.6899999999999999</v>
+        <v>1.24</v>
       </c>
       <c r="G73" t="inlineStr"/>
     </row>
@@ -2886,7 +3106,7 @@
         </is>
       </c>
       <c r="F74" t="n">
-        <v>0.78</v>
+        <v>0.96</v>
       </c>
       <c r="G74" t="inlineStr"/>
     </row>
@@ -2917,7 +3137,7 @@
         </is>
       </c>
       <c r="F75" t="n">
-        <v>0.61</v>
+        <v>2.09</v>
       </c>
       <c r="G75" t="inlineStr"/>
     </row>
@@ -2948,7 +3168,7 @@
         </is>
       </c>
       <c r="F76" t="n">
-        <v>1.09</v>
+        <v>1.21</v>
       </c>
       <c r="G76" t="inlineStr"/>
     </row>
@@ -2979,7 +3199,7 @@
         </is>
       </c>
       <c r="F77" t="n">
-        <v>1.29</v>
+        <v>1.68</v>
       </c>
       <c r="G77" t="inlineStr"/>
     </row>
@@ -3010,7 +3230,7 @@
         </is>
       </c>
       <c r="F78" t="n">
-        <v>0.99</v>
+        <v>1.65</v>
       </c>
       <c r="G78" t="inlineStr"/>
     </row>
@@ -3041,7 +3261,7 @@
         </is>
       </c>
       <c r="F79" t="n">
-        <v>0.78</v>
+        <v>1.51</v>
       </c>
       <c r="G79" t="inlineStr"/>
     </row>
@@ -3072,7 +3292,7 @@
         </is>
       </c>
       <c r="F80" t="n">
-        <v>0.83</v>
+        <v>1.62</v>
       </c>
       <c r="G80" t="inlineStr"/>
     </row>
@@ -3103,7 +3323,7 @@
         </is>
       </c>
       <c r="F81" t="n">
-        <v>1.06</v>
+        <v>2.05</v>
       </c>
       <c r="G81" t="inlineStr"/>
     </row>
@@ -3134,7 +3354,7 @@
         </is>
       </c>
       <c r="F82" t="n">
-        <v>0.87</v>
+        <v>1.89</v>
       </c>
       <c r="G82" t="inlineStr"/>
     </row>
@@ -3165,7 +3385,7 @@
         </is>
       </c>
       <c r="F83" t="n">
-        <v>0.78</v>
+        <v>1.4</v>
       </c>
       <c r="G83" t="inlineStr"/>
     </row>
@@ -3196,7 +3416,7 @@
         </is>
       </c>
       <c r="F84" t="n">
-        <v>0.89</v>
+        <v>16.42</v>
       </c>
       <c r="G84" t="inlineStr"/>
     </row>
@@ -3227,7 +3447,7 @@
         </is>
       </c>
       <c r="F85" t="n">
-        <v>1.1</v>
+        <v>3.16</v>
       </c>
       <c r="G85" t="inlineStr"/>
     </row>
@@ -3258,7 +3478,7 @@
         </is>
       </c>
       <c r="F86" t="n">
-        <v>0.77</v>
+        <v>2</v>
       </c>
       <c r="G86" t="inlineStr"/>
     </row>
@@ -3289,7 +3509,7 @@
         </is>
       </c>
       <c r="F87" t="n">
-        <v>0.76</v>
+        <v>1.68</v>
       </c>
       <c r="G87" t="inlineStr"/>
     </row>
@@ -3320,7 +3540,7 @@
         </is>
       </c>
       <c r="F88" t="n">
-        <v>0.85</v>
+        <v>2.6</v>
       </c>
       <c r="G88" t="inlineStr"/>
     </row>
@@ -3351,7 +3571,7 @@
         </is>
       </c>
       <c r="F89" t="n">
-        <v>0.65</v>
+        <v>1.66</v>
       </c>
       <c r="G89" t="inlineStr"/>
     </row>
@@ -3382,7 +3602,7 @@
         </is>
       </c>
       <c r="F90" t="n">
-        <v>0.8100000000000001</v>
+        <v>7.53</v>
       </c>
       <c r="G90" t="inlineStr"/>
     </row>
@@ -3413,7 +3633,7 @@
         </is>
       </c>
       <c r="F91" t="n">
-        <v>0.91</v>
+        <v>1.69</v>
       </c>
       <c r="G91" t="inlineStr"/>
     </row>
@@ -3444,7 +3664,7 @@
         </is>
       </c>
       <c r="F92" t="n">
-        <v>0.84</v>
+        <v>2.01</v>
       </c>
       <c r="G92" t="inlineStr"/>
     </row>
@@ -3475,7 +3695,7 @@
         </is>
       </c>
       <c r="F93" t="n">
-        <v>0.98</v>
+        <v>3.4</v>
       </c>
       <c r="G93" t="inlineStr"/>
     </row>
@@ -3506,7 +3726,7 @@
         </is>
       </c>
       <c r="F94" t="n">
-        <v>0.67</v>
+        <v>2.88</v>
       </c>
       <c r="G94" t="inlineStr"/>
     </row>
@@ -3537,7 +3757,7 @@
         </is>
       </c>
       <c r="F95" t="n">
-        <v>0.76</v>
+        <v>2.28</v>
       </c>
       <c r="G95" t="inlineStr"/>
     </row>
@@ -3568,7 +3788,7 @@
         </is>
       </c>
       <c r="F96" t="n">
-        <v>0.93</v>
+        <v>5.14</v>
       </c>
       <c r="G96" t="inlineStr"/>
     </row>
@@ -3599,7 +3819,7 @@
         </is>
       </c>
       <c r="F97" t="n">
-        <v>0.79</v>
+        <v>2.3</v>
       </c>
       <c r="G97" t="inlineStr"/>
     </row>
@@ -3630,7 +3850,7 @@
         </is>
       </c>
       <c r="F98" t="n">
-        <v>0.7</v>
+        <v>2.22</v>
       </c>
       <c r="G98" t="inlineStr"/>
     </row>
@@ -3661,7 +3881,7 @@
         </is>
       </c>
       <c r="F99" t="n">
-        <v>0.6899999999999999</v>
+        <v>2.39</v>
       </c>
       <c r="G99" t="inlineStr"/>
     </row>
@@ -3692,7 +3912,7 @@
         </is>
       </c>
       <c r="F100" t="n">
-        <v>0.85</v>
+        <v>1.92</v>
       </c>
       <c r="G100" t="inlineStr"/>
     </row>
@@ -3723,7 +3943,7 @@
         </is>
       </c>
       <c r="F101" t="n">
-        <v>0.77</v>
+        <v>1.07</v>
       </c>
       <c r="G101" t="inlineStr"/>
     </row>
@@ -3754,7 +3974,7 @@
         </is>
       </c>
       <c r="F102" t="n">
-        <v>0.74</v>
+        <v>2.25</v>
       </c>
       <c r="G102" t="inlineStr"/>
     </row>
@@ -3785,7 +4005,7 @@
         </is>
       </c>
       <c r="F103" t="n">
-        <v>0.71</v>
+        <v>7.95</v>
       </c>
       <c r="G103" t="inlineStr"/>
     </row>
@@ -3816,7 +4036,7 @@
         </is>
       </c>
       <c r="F104" t="n">
-        <v>0.67</v>
+        <v>2.01</v>
       </c>
       <c r="G104" t="inlineStr"/>
     </row>
@@ -3909,7 +4129,7 @@
         </is>
       </c>
       <c r="F107" t="n">
-        <v>1.18</v>
+        <v>0.86</v>
       </c>
       <c r="G107" t="inlineStr"/>
     </row>
@@ -3940,7 +4160,7 @@
         </is>
       </c>
       <c r="F108" t="n">
-        <v>4.63</v>
+        <v>2.84</v>
       </c>
       <c r="G108" t="inlineStr"/>
     </row>

</xml_diff>